<commit_message>
Temp Push before merge
</commit_message>
<xml_diff>
--- a/output/forecast.xlsx
+++ b/output/forecast.xlsx
@@ -862,177 +862,177 @@
       <c r="A2"/>
     </row>
     <row r="3">
-      <c r="A3"/>
+      <c r="A3" t="n">
+        <v>0.0119831077049675</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>0.0154386076172396</v>
-      </c>
+      <c r="A4"/>
     </row>
     <row r="5">
       <c r="A5"/>
     </row>
     <row r="6">
-      <c r="A6"/>
+      <c r="A6" t="n">
+        <v>0.0141400253425202</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>0.013659691874553</v>
-      </c>
+      <c r="A7"/>
     </row>
     <row r="8">
       <c r="A8"/>
     </row>
     <row r="9">
-      <c r="A9"/>
+      <c r="A9" t="n">
+        <v>0.0175184853447443</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>0.0147210562606515</v>
-      </c>
+      <c r="A10"/>
     </row>
     <row r="11">
       <c r="A11"/>
     </row>
     <row r="12">
-      <c r="A12"/>
+      <c r="A12" t="n">
+        <v>0.0199046809619106</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>0.0187902053728565</v>
-      </c>
+      <c r="A13"/>
     </row>
     <row r="14">
       <c r="A14"/>
     </row>
     <row r="15">
-      <c r="A15"/>
+      <c r="A15" t="n">
+        <v>0.0190031356862534</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>0.0169553627125188</v>
-      </c>
+      <c r="A16"/>
     </row>
     <row r="17">
       <c r="A17"/>
     </row>
     <row r="18">
-      <c r="A18"/>
+      <c r="A18" t="n">
+        <v>0.0177693024935772</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>0.017702015361575</v>
-      </c>
+      <c r="A19"/>
     </row>
     <row r="20">
       <c r="A20"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="n">
+        <v>0.0166105273562203</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>0.0177996761006313</v>
-      </c>
+      <c r="A22"/>
     </row>
     <row r="23">
       <c r="A23"/>
     </row>
     <row r="24">
-      <c r="A24"/>
+      <c r="A24" t="n">
+        <v>0.0145991900454543</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>0.011582472105742</v>
-      </c>
+      <c r="A25"/>
     </row>
     <row r="26">
       <c r="A26"/>
     </row>
     <row r="27">
-      <c r="A27"/>
+      <c r="A27" t="n">
+        <v>0.00483560602940246</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>0.00778810895998739</v>
-      </c>
+      <c r="A28"/>
     </row>
     <row r="29">
       <c r="A29"/>
     </row>
     <row r="30">
-      <c r="A30"/>
+      <c r="A30" t="n">
+        <v>0.0134257716441824</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
-        <v>0.0147857088629789</v>
-      </c>
+      <c r="A31"/>
     </row>
     <row r="32">
       <c r="A32"/>
     </row>
     <row r="33">
-      <c r="A33"/>
+      <c r="A33" t="n">
+        <v>0.0154768838642043</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>0.0132743582876122</v>
-      </c>
+      <c r="A34"/>
     </row>
     <row r="35">
       <c r="A35"/>
     </row>
     <row r="36">
-      <c r="A36"/>
+      <c r="A36" t="n">
+        <v>-0.0131344227471926</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
-        <v>-0.00309077541782634</v>
-      </c>
+      <c r="A37"/>
     </row>
     <row r="38">
       <c r="A38"/>
     </row>
     <row r="39">
-      <c r="A39"/>
+      <c r="A39" t="n">
+        <v>0.0123049175497882</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
-        <v>0.0108434905333412</v>
-      </c>
+      <c r="A40"/>
     </row>
     <row r="41">
       <c r="A41"/>
     </row>
     <row r="42">
-      <c r="A42"/>
+      <c r="A42" t="n">
+        <v>0.0116115724772109</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
-        <v>0.010683368843575</v>
-      </c>
+      <c r="A43"/>
     </row>
     <row r="44">
       <c r="A44"/>
     </row>
     <row r="45">
-      <c r="A45"/>
+      <c r="A45" t="n">
+        <v>0.00992850569382401</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
-        <v>0.00855271355228642</v>
-      </c>
+      <c r="A46"/>
     </row>
     <row r="47">
       <c r="A47"/>
     </row>
     <row r="48">
-      <c r="A48"/>
+      <c r="A48" t="n">
+        <v>0.0119905577925275</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
-        <v>0.0171450667313933</v>
-      </c>
+      <c r="A49"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1052,177 +1052,177 @@
       <c r="A2"/>
     </row>
     <row r="3">
-      <c r="A3"/>
+      <c r="A3" t="n">
+        <v>0.0142854486517984</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>0.0117326209820302</v>
-      </c>
+      <c r="A4"/>
     </row>
     <row r="5">
       <c r="A5"/>
     </row>
     <row r="6">
-      <c r="A6"/>
+      <c r="A6" t="n">
+        <v>0.0150314772321275</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>0.0108960504825199</v>
-      </c>
+      <c r="A7"/>
     </row>
     <row r="8">
       <c r="A8"/>
     </row>
     <row r="9">
-      <c r="A9"/>
+      <c r="A9" t="n">
+        <v>0.0156242751154899</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>0.0161802896959579</v>
-      </c>
+      <c r="A10"/>
     </row>
     <row r="11">
       <c r="A11"/>
     </row>
     <row r="12">
-      <c r="A12"/>
+      <c r="A12" t="n">
+        <v>0.00944838653556705</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>0.018865813994737</v>
-      </c>
+      <c r="A13"/>
     </row>
     <row r="14">
       <c r="A14"/>
     </row>
     <row r="15">
-      <c r="A15"/>
+      <c r="A15" t="n">
+        <v>0.00699843935567633</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>0.0194895834451105</v>
-      </c>
+      <c r="A16"/>
     </row>
     <row r="17">
       <c r="A17"/>
     </row>
     <row r="18">
-      <c r="A18"/>
+      <c r="A18" t="n">
+        <v>0.0162932810153103</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>0.0181146635128779</v>
-      </c>
+      <c r="A19"/>
     </row>
     <row r="20">
       <c r="A20"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="n">
+        <v>0.0158419786947058</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>0.0171766330360351</v>
-      </c>
+      <c r="A22"/>
     </row>
     <row r="23">
       <c r="A23"/>
     </row>
     <row r="24">
-      <c r="A24"/>
+      <c r="A24" t="n">
+        <v>0.00650668343248845</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>0.0141973969864204</v>
-      </c>
+      <c r="A25"/>
     </row>
     <row r="26">
       <c r="A26"/>
     </row>
     <row r="27">
-      <c r="A27"/>
+      <c r="A27" t="n">
+        <v>-0.0018174553401396</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>0.00865166573210851</v>
-      </c>
+      <c r="A28"/>
     </row>
     <row r="29">
       <c r="A29"/>
     </row>
     <row r="30">
-      <c r="A30"/>
+      <c r="A30" t="n">
+        <v>0.0116869810065715</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
-        <v>0.0141642234284751</v>
-      </c>
+      <c r="A31"/>
     </row>
     <row r="32">
       <c r="A32"/>
     </row>
     <row r="33">
-      <c r="A33"/>
+      <c r="A33" t="n">
+        <v>0.0148103519240211</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>0.015211729534928</v>
-      </c>
+      <c r="A34"/>
     </row>
     <row r="35">
       <c r="A35"/>
     </row>
     <row r="36">
-      <c r="A36"/>
+      <c r="A36" t="n">
+        <v>-0.00658036484898109</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
-        <v>-0.00936389661164536</v>
-      </c>
+      <c r="A37"/>
     </row>
     <row r="38">
       <c r="A38"/>
     </row>
     <row r="39">
-      <c r="A39"/>
+      <c r="A39" t="n">
+        <v>0.00872296365314064</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
-        <v>0.00943938906387804</v>
-      </c>
+      <c r="A40"/>
     </row>
     <row r="41">
       <c r="A41"/>
     </row>
     <row r="42">
-      <c r="A42"/>
+      <c r="A42" t="n">
+        <v>0.0107802660902604</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
-        <v>0.0106183406935087</v>
-      </c>
+      <c r="A43"/>
     </row>
     <row r="44">
       <c r="A44"/>
     </row>
     <row r="45">
-      <c r="A45"/>
+      <c r="A45" t="n">
+        <v>0.0137436803366078</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
-        <v>0.00768883773290075</v>
-      </c>
+      <c r="A46"/>
     </row>
     <row r="47">
       <c r="A47"/>
     </row>
     <row r="48">
-      <c r="A48"/>
+      <c r="A48" t="n">
+        <v>0.00939744059426976</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
-        <v>0.0127475748282161</v>
-      </c>
+      <c r="A49"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1245,174 +1245,172 @@
       <c r="A3"/>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>0.00224425051409125</v>
-      </c>
+      <c r="A4"/>
     </row>
     <row r="5">
       <c r="A5"/>
     </row>
     <row r="6">
-      <c r="A6"/>
+      <c r="A6" t="n">
+        <v>0.0151154123346442</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>0.0118035666760139</v>
-      </c>
+      <c r="A7"/>
     </row>
     <row r="8">
       <c r="A8"/>
     </row>
     <row r="9">
-      <c r="A9"/>
+      <c r="A9" t="n">
+        <v>0.012424631948694</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>0.0133111145982076</v>
-      </c>
+      <c r="A10"/>
     </row>
     <row r="11">
       <c r="A11"/>
     </row>
     <row r="12">
-      <c r="A12"/>
+      <c r="A12" t="n">
+        <v>0.0119942287720807</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>0.0115094421321763</v>
-      </c>
+      <c r="A13"/>
     </row>
     <row r="14">
       <c r="A14"/>
     </row>
     <row r="15">
-      <c r="A15"/>
+      <c r="A15" t="n">
+        <v>0.0148578401410816</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>0.00210185036912208</v>
-      </c>
+      <c r="A16"/>
     </row>
     <row r="17">
       <c r="A17"/>
     </row>
     <row r="18">
-      <c r="A18"/>
+      <c r="A18" t="n">
+        <v>0.0178127339713151</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>0.0157817199394054</v>
-      </c>
+      <c r="A19"/>
     </row>
     <row r="20">
       <c r="A20"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="n">
+        <v>0.0156071313330172</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>0.0160173225725187</v>
-      </c>
+      <c r="A22"/>
     </row>
     <row r="23">
       <c r="A23"/>
     </row>
     <row r="24">
-      <c r="A24"/>
+      <c r="A24" t="n">
+        <v>0.0167349508545653</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>0.00649367828427385</v>
-      </c>
+      <c r="A25"/>
     </row>
     <row r="26">
       <c r="A26"/>
     </row>
     <row r="27">
-      <c r="A27"/>
+      <c r="A27" t="n">
+        <v>0.0104175961997972</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>-0.00656147880518532</v>
-      </c>
+      <c r="A28"/>
     </row>
     <row r="29">
       <c r="A29"/>
     </row>
     <row r="30">
-      <c r="A30"/>
+      <c r="A30" t="n">
+        <v>0.0123851371020795</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
-        <v>0.0120540133077287</v>
-      </c>
+      <c r="A31"/>
     </row>
     <row r="32">
       <c r="A32"/>
     </row>
     <row r="33">
-      <c r="A33"/>
+      <c r="A33" t="n">
+        <v>0.013829324462614</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>0.0139675151322535</v>
-      </c>
+      <c r="A34"/>
     </row>
     <row r="35">
       <c r="A35"/>
     </row>
     <row r="36">
-      <c r="A36"/>
+      <c r="A36" t="n">
+        <v>0.0108500204293118</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
-        <v>-0.00163609476351289</v>
-      </c>
+      <c r="A37"/>
     </row>
     <row r="38">
       <c r="A38"/>
     </row>
     <row r="39">
-      <c r="A39"/>
+      <c r="A39" t="n">
+        <v>0.0102656242615928</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
-        <v>0.00368925767125473</v>
-      </c>
+      <c r="A40"/>
     </row>
     <row r="41">
       <c r="A41"/>
     </row>
     <row r="42">
-      <c r="A42"/>
+      <c r="A42" t="n">
+        <v>0.0115218802883047</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
-        <v>0.00990661223353952</v>
-      </c>
+      <c r="A43"/>
     </row>
     <row r="44">
       <c r="A44"/>
     </row>
     <row r="45">
-      <c r="A45"/>
+      <c r="A45" t="n">
+        <v>0.0106530533734221</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
-        <v>0.0129939038329548</v>
-      </c>
+      <c r="A46"/>
     </row>
     <row r="47">
       <c r="A47"/>
     </row>
     <row r="48">
-      <c r="A48"/>
+      <c r="A48" t="n">
+        <v>0.00974799948317735</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
-        <v>0.0091358992610698</v>
-      </c>
+      <c r="A49"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>